<commit_message>
chore: project update (#6)
* project update

* up

* up

* up

* up

* up

* up

* up

* up

* up

* Updated logo

* up

* updated tests

* Updated CI

* up

* up

* up

* up

* up

* up

* up
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="simple" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="complex" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Row1Col1</t>
+          <t>ABC</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -441,7 +442,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Row2Col1</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -451,7 +452,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MergedValue</t>
+          <t>Merged value</t>
         </is>
       </c>
     </row>
@@ -462,4 +463,225 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Financial Report 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12000.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>15000.75</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18000.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>9500</v>
+      </c>
+      <c r="C5" t="n">
+        <v>11000.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10500.2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12000.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>14000.1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>16500.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>21000.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C7" t="n">
+        <v>12500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14500</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>SUM(B4:B7)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>SUM(C4:C7)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>SUM(D4:D7)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUM(E4:E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2023-01-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2021-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Confidential - Internal Use Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B14:D15"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implemented more APIs (#9)
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -414,18 +414,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Header1</t>
+          <t>Header #1</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Header2</t>
+          <t>Header #2</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Header #3</t>
         </is>
       </c>
     </row>
@@ -438,6 +443,11 @@
       <c r="B2" t="n">
         <v>123.45</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -448,6 +458,11 @@
       <c r="B3" t="n">
         <v>678</v>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -455,8 +470,19 @@
           <t>Merged value</t>
         </is>
       </c>
-    </row>
-    <row r="5"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Charlie</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A4:B5"/>

</xml_diff>

<commit_message>
Added support for Date / DateTime cells
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -98,11 +98,11 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -733,10 +733,8 @@
       <c r="C11" t="b">
         <v>1</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2023-01-15</t>
-        </is>
+      <c r="D11" s="1" t="n">
+        <v>44941</v>
       </c>
     </row>
     <row r="12">
@@ -753,10 +751,8 @@
       <c r="C12" t="b">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2021-06-01</t>
-        </is>
+      <c r="D12" s="1" t="n">
+        <v>44348</v>
       </c>
     </row>
     <row r="14">
@@ -846,28 +842,28 @@
       </c>
     </row>
     <row r="7" ht="35" customHeight="1">
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Financial Report</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="1" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="1" t="n">
         <v>46196</v>
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Fiscal Year</t>
         </is>

</xml_diff>

<commit_message>
feat: support new features (#15)
Added support for Date / DateTime cells
Added support for nested cell group matching
Added support for greedy/lazy matching
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="simple" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="complex" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="multi-tables" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +29,59 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000080"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+        <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +96,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,10 +733,8 @@
       <c r="C11" t="b">
         <v>1</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2023-01-15</t>
-        </is>
+      <c r="D11" s="1" t="n">
+        <v>44941</v>
       </c>
     </row>
     <row r="12">
@@ -689,10 +751,8 @@
       <c r="C12" t="b">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2021-06-01</t>
-        </is>
+      <c r="D12" s="1" t="n">
+        <v>44348</v>
       </c>
     </row>
     <row r="14">
@@ -710,4 +770,626 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" hidden="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>INT-CODE-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" hidden="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>INT-CODE-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" hidden="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>INT-CODE-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" hidden="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>INT-CODE-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INT-CODE-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="35" customHeight="1">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Financial Report</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Fiscal Year</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Product A</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>427</v>
+      </c>
+      <c r="D15" t="n">
+        <v>147</v>
+      </c>
+      <c r="E15" t="n">
+        <v>122</v>
+      </c>
+      <c r="F15" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>240</v>
+      </c>
+      <c r="D16" t="n">
+        <v>215</v>
+      </c>
+      <c r="E16" t="n">
+        <v>224</v>
+      </c>
+      <c r="F16" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>477</v>
+      </c>
+      <c r="D17" t="n">
+        <v>142</v>
+      </c>
+      <c r="E17" t="n">
+        <v>456</v>
+      </c>
+      <c r="F17" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C18" s="7">
+        <f>SUM(C15:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="7">
+        <f>SUM(D15:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="7">
+        <f>SUM(E15:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="7">
+        <f>SUM(F15:F17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Product A</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>379</v>
+      </c>
+      <c r="D23" t="n">
+        <v>134</v>
+      </c>
+      <c r="E23" t="n">
+        <v>412</v>
+      </c>
+      <c r="F23" t="n">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>116</v>
+      </c>
+      <c r="D24" t="n">
+        <v>105</v>
+      </c>
+      <c r="E24" t="n">
+        <v>157</v>
+      </c>
+      <c r="F24" t="n">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>219</v>
+      </c>
+      <c r="D25" t="n">
+        <v>348</v>
+      </c>
+      <c r="E25" t="n">
+        <v>418</v>
+      </c>
+      <c r="F25" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Product D</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>387</v>
+      </c>
+      <c r="D26" t="n">
+        <v>191</v>
+      </c>
+      <c r="E26" t="n">
+        <v>476</v>
+      </c>
+      <c r="F26" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C27" s="7">
+        <f>SUM(C23:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="7">
+        <f>SUM(D23:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="7">
+        <f>SUM(E23:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="7">
+        <f>SUM(F23:F26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F30" s="5" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Product A</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>459</v>
+      </c>
+      <c r="D32" t="n">
+        <v>369</v>
+      </c>
+      <c r="E32" t="n">
+        <v>324</v>
+      </c>
+      <c r="F32" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>329</v>
+      </c>
+      <c r="D33" t="n">
+        <v>391</v>
+      </c>
+      <c r="E33" t="n">
+        <v>252</v>
+      </c>
+      <c r="F33" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C34" s="7">
+        <f>SUM(C32:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="7">
+        <f>SUM(D32:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="7">
+        <f>SUM(E32:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="7">
+        <f>SUM(F32:F33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F37" s="5" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Product A</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>103</v>
+      </c>
+      <c r="D39" t="n">
+        <v>478</v>
+      </c>
+      <c r="E39" t="n">
+        <v>522</v>
+      </c>
+      <c r="F39" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>457</v>
+      </c>
+      <c r="D40" t="n">
+        <v>306</v>
+      </c>
+      <c r="E40" t="n">
+        <v>284</v>
+      </c>
+      <c r="F40" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>179</v>
+      </c>
+      <c r="D41" t="n">
+        <v>200</v>
+      </c>
+      <c r="E41" t="n">
+        <v>500</v>
+      </c>
+      <c r="F41" t="n">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C42" s="7">
+        <f>SUM(C39:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="7">
+        <f>SUM(D39:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="7">
+        <f>SUM(E39:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="7">
+        <f>SUM(F39:F41)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="E21:F21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add tutorial for sub headers and footers
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -10,6 +10,7 @@
     <sheet name="simple" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="complex" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="multi-tables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="sub-sections" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +58,19 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +95,12 @@
         <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -96,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -111,6 +129,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1392,4 +1434,310 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Spent</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Development Department</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D4" s="11">
+        <f>B4-C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>75000</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D5" s="11">
+        <f>B5-C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D6" s="11">
+        <f>B6-C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="13">
+        <f>SUM(B4:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="13">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="13">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Marketing Department</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Campaign X</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>18000</v>
+      </c>
+      <c r="D9" s="11">
+        <f>B9-C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Campaign Y</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>16000</v>
+      </c>
+      <c r="D10" s="11">
+        <f>B10-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B11" s="13">
+        <f>SUM(B9:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="13">
+        <f>SUM(C9:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>SUM(D9:D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Sales Department</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Direct Sales</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>95000</v>
+      </c>
+      <c r="D13" s="11">
+        <f>B13-C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Online Sales</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D14" s="11">
+        <f>B14-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Partner Channels</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>62000</v>
+      </c>
+      <c r="D15" s="11">
+        <f>B15-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Retail Outlets</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D16" s="11">
+        <f>B16-C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B17" s="13">
+        <f>SUM(B13:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="13">
+        <f>SUM(C13:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>SUM(D13:D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>B7+B11+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>C7+C11+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>D7+D11+D17</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add tutorial for sub headers and footers (#44)
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -10,6 +10,7 @@
     <sheet name="simple" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="complex" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="multi-tables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="sub-sections" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +58,19 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +95,12 @@
         <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -96,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -111,6 +129,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1392,4 +1434,310 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Spent</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Development Department</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D4" s="11">
+        <f>B4-C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>75000</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D5" s="11">
+        <f>B5-C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D6" s="11">
+        <f>B6-C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="13">
+        <f>SUM(B4:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="13">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="13">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Marketing Department</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Campaign X</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>18000</v>
+      </c>
+      <c r="D9" s="11">
+        <f>B9-C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Campaign Y</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>16000</v>
+      </c>
+      <c r="D10" s="11">
+        <f>B10-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B11" s="13">
+        <f>SUM(B9:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="13">
+        <f>SUM(C9:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>SUM(D9:D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Sales Department</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Direct Sales</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>95000</v>
+      </c>
+      <c r="D13" s="11">
+        <f>B13-C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Online Sales</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D14" s="11">
+        <f>B14-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Partner Channels</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>62000</v>
+      </c>
+      <c r="D15" s="11">
+        <f>B15-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Retail Outlets</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D16" s="11">
+        <f>B16-C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B17" s="13">
+        <f>SUM(B13:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="13">
+        <f>SUM(C13:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>SUM(D13:D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>B7+B11+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>C7+C11+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>D7+D11+D17</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>